<commit_message>
update: Chee 52,564 steps (week of 1 Jun) = Tier 1, total now 24pts
</commit_message>
<xml_diff>
--- a/Reports/Members/Chee_Activity_Report.xlsx
+++ b/Reports/Members/Chee_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,6 +506,53 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>6/7/2026 21:02:41</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chee</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>52,564</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Healthy 365</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -589,7 +636,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>69621</v>
+        <v>122185</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -627,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>69621</v>
+        <v>122185</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>

</xml_diff>